<commit_message>
Marketplace: append '- Marketplace <Year>' suffix to all plan names (SOB + EOC); related config, page, spec and data updates
Aligns Plans workbook titles with UI card display change and disables CA SOB rows now that SOB is not offered in the Category filter.
</commit_message>
<xml_diff>
--- a/data/marketplace/MarketplaceBrochureFormularyData.xlsx
+++ b/data/marketplace/MarketplaceBrochureFormularyData.xlsx
@@ -8,20 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molinahealthcare-my.sharepoint.com/personal/naresh_jangid_molinahealthcare_com/Documents/Automation/molina_automation/marketplace/data/marketplace/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_C8CED50611474A6E54521311C477A1F5D0A88FCC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8782B94-3435-4737-950D-92CF8A9F3C2B}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_00DF86192339FA6CDC610236489088D5A02C51E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA811E6E-F4FF-48E2-B8B3-3FAFC50D91F0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BrochureFormulary" sheetId="1" r:id="rId1"/>
-    <sheet name="Settings" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="112">
   <si>
     <t>Run</t>
   </si>
@@ -65,6 +64,9 @@
     <t>MemberBrochure_ES_URL</t>
   </si>
   <si>
+    <t>BrokerBrochure_Search</t>
+  </si>
+  <si>
     <t>BrokerBrochure_EN_Name</t>
   </si>
   <si>
@@ -107,10 +109,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/ca/materials/formulary/2027/spanish/CAFormulary27.pdf</t>
   </si>
   <si>
-    <t>CAMBRBrochure27</t>
-  </si>
-  <si>
-    <t>CAMBRBrochure27.pdf</t>
+    <t>CA Plan Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/ca/materials/brochure/2027/english/CAMBRBrochure27.pdf</t>
@@ -119,7 +118,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/ca/materials/brochure/2027/spanish/CAMBRBrochure27.pdf</t>
   </si>
   <si>
-    <t>CABrochure27.pdf</t>
+    <t>CA Broker Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/ca/materials/brochure/2027/english/CABrochure27.pdf</t>
@@ -152,10 +151,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/id/materials/formulary/2027/spanish/IDFormulary27.pdf</t>
   </si>
   <si>
-    <t>IDMBRBrochure27</t>
-  </si>
-  <si>
-    <t>IDMBRBrochure27.pdf</t>
+    <t>ID Plan Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/id/materials/brochure/2027/english/IDMBRBrochure27.pdf</t>
@@ -164,7 +160,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/id/materials/brochure/2027/spanish/IDMBRBrochure27.pdf</t>
   </si>
   <si>
-    <t>IDBrochure27.pdf</t>
+    <t>ID Broker Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/id/materials/brochure/2027/english/IDBrochure27.pdf</t>
@@ -194,10 +190,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/formulary/2027/spanish/NMFormulary27.pdf</t>
   </si>
   <si>
-    <t>NMMBRBrochure27</t>
-  </si>
-  <si>
-    <t>NMMBRBrochure27.pdf</t>
+    <t>NM Plan Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/brochure/2027/english/NMMBRBrochure27.pdf</t>
@@ -206,7 +199,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/brochure/2027/spanish/NMMBRBrochure27.pdf</t>
   </si>
   <si>
-    <t>NMBrochure27.pdf</t>
+    <t>NM Broker Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/brochure/2027/english/NMBrochure27.pdf</t>
@@ -236,10 +229,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/formulary/2027/spanish/NVFormulary27.pdf</t>
   </si>
   <si>
-    <t>NVMBRBrochure27</t>
-  </si>
-  <si>
-    <t>NVMBRBrochure27.pdf</t>
+    <t>NV Plan Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/brochure/2027/english/NVMBRBrochure27.pdf</t>
@@ -248,7 +238,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/brochure/2027/spanish/NVMBRBrochure27.pdf</t>
   </si>
   <si>
-    <t>NVBrochure27.pdf</t>
+    <t>NV Broker Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/brochure/2027/english/NVBrochure27.pdf</t>
@@ -278,10 +268,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/formulary/2027/spanish/TXFormulary27.pdf</t>
   </si>
   <si>
-    <t>TXMBRBrochure27</t>
-  </si>
-  <si>
-    <t>TXMBRBrochure27.pdf</t>
+    <t>TX Plan Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/brochure/2027/english/TXMBRBrochure27.pdf</t>
@@ -290,7 +277,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/brochure/2027/spanish/TXMBRBrochure27.pdf</t>
   </si>
   <si>
-    <t>TXBrochure27.pdf</t>
+    <t>TX Broker Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/brochure/2027/english/TXBrochure27.pdf</t>
@@ -308,10 +295,7 @@
     <t>TX-OX</t>
   </si>
   <si>
-    <t>TXOXMBRBrochure27</t>
-  </si>
-  <si>
-    <t>TXOXMBRBrochure27.pdf</t>
+    <t>TX Off Exchange Plan Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/brochure/2027/english/TXOXMBRBrochure27.pdf</t>
@@ -320,7 +304,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/brochure/2027/spanish/TXOXMBRBrochure27.pdf</t>
   </si>
   <si>
-    <t>TXOXBrochure27.pdf</t>
+    <t>TX Off Exchange Broker Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/brochure/2027/english/TXOXBrochure27.pdf</t>
@@ -350,10 +334,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/formulary/2027/spanish/WAFormulary27.pdf</t>
   </si>
   <si>
-    <t>WAMBRBrochure27</t>
-  </si>
-  <si>
-    <t>WAMBRBrochure27.pdf</t>
+    <t>WA Plan Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/brochure/2027/english/WAMBRBrochure27.pdf</t>
@@ -362,7 +343,7 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/brochure/2027/spanish/WAMBRBrochure27.pdf</t>
   </si>
   <si>
-    <t>WABrochure27.pdf</t>
+    <t>WA Broker Brochure</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/brochure/2027/english/WABrochure27.pdf</t>
@@ -372,84 +353,6 @@
   </si>
   <si>
     <t>MolinaHealthcare.com/WAFormulary27</t>
-  </si>
-  <si>
-    <t>Key</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>AppUrl</t>
-  </si>
-  <si>
-    <t>https://uat-pws.molinahealthcare.com/</t>
-  </si>
-  <si>
-    <t>Landing page for the suite</t>
-  </si>
-  <si>
-    <t>Audience</t>
-  </si>
-  <si>
-    <t>Marketplace</t>
-  </si>
-  <si>
-    <t>Audience filter label</t>
-  </si>
-  <si>
-    <t>FormularyCategory</t>
-  </si>
-  <si>
-    <t>Formulary and Drug Lists</t>
-  </si>
-  <si>
-    <t>Category filter label for Formulary pass</t>
-  </si>
-  <si>
-    <t>BrochureCategory</t>
-  </si>
-  <si>
-    <t>Member Handbooks and Coverage</t>
-  </si>
-  <si>
-    <t>Category filter label for Member + Broker Brochure pass</t>
-  </si>
-  <si>
-    <t>SourceHost</t>
-  </si>
-  <si>
-    <t>www.molinahealthcare.com</t>
-  </si>
-  <si>
-    <t>Host in sheet URLs (prod)</t>
-  </si>
-  <si>
-    <t>TargetHost</t>
-  </si>
-  <si>
-    <t>uat-pws.molinahealthcare.com</t>
-  </si>
-  <si>
-    <t>Host to rewrite to at test time</t>
-  </si>
-  <si>
-    <t>Languages</t>
-  </si>
-  <si>
-    <t>en,es</t>
-  </si>
-  <si>
-    <t>Comma-separated site-language passes</t>
-  </si>
-  <si>
-    <t>BrokerEnabled</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>Set to false to skip Broker Brochure step</t>
   </si>
   <si>
     <t>N</t>
@@ -829,8 +732,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:U8"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.796875" customWidth="1"/>
     <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
@@ -840,13 +743,13 @@
     <col min="8" max="9" width="110.796875" customWidth="1"/>
     <col min="10" max="12" width="30.796875" customWidth="1"/>
     <col min="13" max="14" width="110.796875" customWidth="1"/>
-    <col min="15" max="16" width="30.796875" customWidth="1"/>
-    <col min="17" max="18" width="110.796875" customWidth="1"/>
-    <col min="19" max="19" width="40.796875" customWidth="1"/>
-    <col min="20" max="20" width="46.796875" customWidth="1"/>
+    <col min="15" max="17" width="30.796875" customWidth="1"/>
+    <col min="18" max="19" width="110.796875" customWidth="1"/>
+    <col min="20" max="20" width="40.796875" customWidth="1"/>
+    <col min="21" max="21" width="46.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -907,37 +810,40 @@
       <c r="T1" t="s">
         <v>19</v>
       </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>143</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K2" t="s">
         <v>29</v>
@@ -958,21 +864,24 @@
         <v>32</v>
       </c>
       <c r="Q2" t="s">
+        <v>32</v>
+      </c>
+      <c r="R2" t="s">
         <v>33</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>34</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>35</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="B3" t="s">
         <v>37</v>
@@ -981,7 +890,7 @@
         <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" t="s">
         <v>39</v>
@@ -1002,234 +911,246 @@
         <v>43</v>
       </c>
       <c r="K3" t="s">
+        <v>43</v>
+      </c>
+      <c r="L3" t="s">
+        <v>43</v>
+      </c>
+      <c r="M3" t="s">
         <v>44</v>
       </c>
-      <c r="L3" t="s">
-        <v>44</v>
-      </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>45</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>46</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>46</v>
+      </c>
+      <c r="R3" t="s">
         <v>47</v>
       </c>
-      <c r="P3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q3" t="s">
+      <c r="S3" t="s">
         <v>48</v>
       </c>
-      <c r="R3" t="s">
+      <c r="T3" t="s">
         <v>49</v>
       </c>
-      <c r="S3" t="s">
+      <c r="U3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" t="s">
         <v>50</v>
       </c>
-      <c r="T3" t="s">
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G4" t="s">
+        <v>53</v>
+      </c>
+      <c r="H4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" t="s">
+        <v>56</v>
+      </c>
+      <c r="K4" t="s">
+        <v>56</v>
+      </c>
+      <c r="L4" t="s">
+        <v>56</v>
+      </c>
+      <c r="M4" t="s">
+        <v>57</v>
+      </c>
+      <c r="N4" t="s">
+        <v>58</v>
+      </c>
+      <c r="O4" t="s">
+        <v>59</v>
+      </c>
+      <c r="P4" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>59</v>
+      </c>
+      <c r="R4" t="s">
+        <v>60</v>
+      </c>
+      <c r="S4" t="s">
+        <v>61</v>
+      </c>
+      <c r="T4" t="s">
+        <v>62</v>
+      </c>
+      <c r="U4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" t="s">
-        <v>53</v>
-      </c>
-      <c r="F4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G4" t="s">
-        <v>54</v>
-      </c>
-      <c r="H4" t="s">
-        <v>55</v>
-      </c>
-      <c r="I4" t="s">
-        <v>56</v>
-      </c>
-      <c r="J4" t="s">
-        <v>57</v>
-      </c>
-      <c r="K4" t="s">
-        <v>58</v>
-      </c>
-      <c r="L4" t="s">
-        <v>58</v>
-      </c>
-      <c r="M4" t="s">
-        <v>59</v>
-      </c>
-      <c r="N4" t="s">
-        <v>60</v>
-      </c>
-      <c r="O4" t="s">
-        <v>61</v>
-      </c>
-      <c r="P4" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>62</v>
-      </c>
-      <c r="R4" t="s">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
         <v>63</v>
       </c>
-      <c r="S4" t="s">
+      <c r="C5" t="s">
         <v>64</v>
       </c>
-      <c r="T4" t="s">
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J5" t="s">
+        <v>69</v>
+      </c>
+      <c r="K5" t="s">
+        <v>69</v>
+      </c>
+      <c r="L5" t="s">
+        <v>69</v>
+      </c>
+      <c r="M5" t="s">
+        <v>70</v>
+      </c>
+      <c r="N5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O5" t="s">
+        <v>72</v>
+      </c>
+      <c r="P5" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>72</v>
+      </c>
+      <c r="R5" t="s">
+        <v>73</v>
+      </c>
+      <c r="S5" t="s">
+        <v>74</v>
+      </c>
+      <c r="T5" t="s">
+        <v>75</v>
+      </c>
+      <c r="U5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>67</v>
-      </c>
-      <c r="F5" t="s">
-        <v>68</v>
-      </c>
-      <c r="G5" t="s">
-        <v>68</v>
-      </c>
-      <c r="H5" t="s">
-        <v>69</v>
-      </c>
-      <c r="I5" t="s">
-        <v>70</v>
-      </c>
-      <c r="J5" t="s">
-        <v>71</v>
-      </c>
-      <c r="K5" t="s">
-        <v>72</v>
-      </c>
-      <c r="L5" t="s">
-        <v>72</v>
-      </c>
-      <c r="M5" t="s">
-        <v>73</v>
-      </c>
-      <c r="N5" t="s">
-        <v>74</v>
-      </c>
-      <c r="O5" t="s">
-        <v>75</v>
-      </c>
-      <c r="P5" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q5" t="s">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" t="s">
         <v>76</v>
       </c>
-      <c r="R5" t="s">
+      <c r="C6" t="s">
         <v>77</v>
       </c>
-      <c r="S5" t="s">
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
         <v>78</v>
       </c>
-      <c r="T5" t="s">
+      <c r="F6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G6" t="s">
+        <v>79</v>
+      </c>
+      <c r="H6" t="s">
+        <v>80</v>
+      </c>
+      <c r="I6" t="s">
+        <v>81</v>
+      </c>
+      <c r="J6" t="s">
+        <v>82</v>
+      </c>
+      <c r="K6" t="s">
+        <v>82</v>
+      </c>
+      <c r="L6" t="s">
+        <v>82</v>
+      </c>
+      <c r="M6" t="s">
+        <v>83</v>
+      </c>
+      <c r="N6" t="s">
+        <v>84</v>
+      </c>
+      <c r="O6" t="s">
+        <v>85</v>
+      </c>
+      <c r="P6" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>85</v>
+      </c>
+      <c r="R6" t="s">
+        <v>86</v>
+      </c>
+      <c r="S6" t="s">
+        <v>87</v>
+      </c>
+      <c r="T6" t="s">
+        <v>88</v>
+      </c>
+      <c r="U6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>143</v>
-      </c>
-      <c r="B6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" t="s">
-        <v>81</v>
-      </c>
-      <c r="F6" t="s">
-        <v>82</v>
-      </c>
-      <c r="G6" t="s">
-        <v>82</v>
-      </c>
-      <c r="H6" t="s">
-        <v>83</v>
-      </c>
-      <c r="I6" t="s">
-        <v>84</v>
-      </c>
-      <c r="J6" t="s">
-        <v>85</v>
-      </c>
-      <c r="K6" t="s">
-        <v>86</v>
-      </c>
-      <c r="L6" t="s">
-        <v>86</v>
-      </c>
-      <c r="M6" t="s">
-        <v>87</v>
-      </c>
-      <c r="N6" t="s">
-        <v>88</v>
-      </c>
-      <c r="O6" t="s">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" t="s">
         <v>89</v>
       </c>
-      <c r="P6" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q6" t="s">
+      <c r="C7" t="s">
         <v>90</v>
       </c>
-      <c r="R6" t="s">
-        <v>91</v>
-      </c>
-      <c r="S6" t="s">
-        <v>92</v>
-      </c>
-      <c r="T6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>143</v>
-      </c>
-      <c r="B7" t="s">
-        <v>93</v>
-      </c>
-      <c r="C7" t="s">
-        <v>94</v>
-      </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7" t="s">
         <v>36</v>
@@ -1247,222 +1168,117 @@
         <v>36</v>
       </c>
       <c r="J7" t="s">
+        <v>91</v>
+      </c>
+      <c r="K7" t="s">
+        <v>91</v>
+      </c>
+      <c r="L7" t="s">
+        <v>91</v>
+      </c>
+      <c r="M7" t="s">
+        <v>92</v>
+      </c>
+      <c r="N7" t="s">
+        <v>93</v>
+      </c>
+      <c r="O7" t="s">
+        <v>94</v>
+      </c>
+      <c r="P7" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>94</v>
+      </c>
+      <c r="R7" t="s">
         <v>95</v>
       </c>
-      <c r="K7" t="s">
+      <c r="S7" t="s">
         <v>96</v>
       </c>
-      <c r="L7" t="s">
-        <v>96</v>
-      </c>
-      <c r="M7" t="s">
+      <c r="T7" t="s">
+        <v>36</v>
+      </c>
+      <c r="U7" t="s">
         <v>97</v>
       </c>
-      <c r="N7" t="s">
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B8" t="s">
         <v>98</v>
       </c>
-      <c r="O7" t="s">
+      <c r="C8" t="s">
         <v>99</v>
       </c>
-      <c r="P7" t="s">
-        <v>99</v>
-      </c>
-      <c r="Q7" t="s">
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" t="s">
         <v>100</v>
       </c>
-      <c r="R7" t="s">
+      <c r="F8" t="s">
         <v>101</v>
       </c>
-      <c r="S7" t="s">
-        <v>36</v>
-      </c>
-      <c r="T7" t="s">
+      <c r="G8" t="s">
+        <v>101</v>
+      </c>
+      <c r="H8" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="8" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>143</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="I8" t="s">
         <v>103</v>
       </c>
-      <c r="C8" t="s">
+      <c r="J8" t="s">
         <v>104</v>
       </c>
-      <c r="D8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="K8" t="s">
+        <v>104</v>
+      </c>
+      <c r="L8" t="s">
+        <v>104</v>
+      </c>
+      <c r="M8" t="s">
         <v>105</v>
       </c>
-      <c r="F8" t="s">
+      <c r="N8" t="s">
         <v>106</v>
       </c>
-      <c r="G8" t="s">
-        <v>106</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="O8" t="s">
         <v>107</v>
       </c>
-      <c r="I8" t="s">
+      <c r="P8" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>107</v>
+      </c>
+      <c r="R8" t="s">
         <v>108</v>
       </c>
-      <c r="J8" t="s">
+      <c r="S8" t="s">
         <v>109</v>
       </c>
-      <c r="K8" t="s">
+      <c r="T8" t="s">
         <v>110</v>
       </c>
-      <c r="L8" t="s">
-        <v>110</v>
-      </c>
-      <c r="M8" t="s">
-        <v>111</v>
-      </c>
-      <c r="N8" t="s">
-        <v>112</v>
-      </c>
-      <c r="O8" t="s">
-        <v>113</v>
-      </c>
-      <c r="P8" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>114</v>
-      </c>
-      <c r="R8" t="s">
-        <v>115</v>
-      </c>
-      <c r="S8" t="s">
-        <v>116</v>
-      </c>
-      <c r="T8" t="s">
+      <c r="U8" t="s">
         <v>36</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:T1 A3:T5 B2:T2 B7:T8 B6:T6" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:U1 B4:U8 B3:U3 B2:U2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="22.796875" customWidth="1"/>
-    <col min="2" max="2" width="50.796875" customWidth="1"/>
-    <col min="3" max="3" width="60.796875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B1" t="s">
-        <v>118</v>
-      </c>
-      <c r="C1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>122</v>
-      </c>
-      <c r="B3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B4" t="s">
-        <v>126</v>
-      </c>
-      <c r="C4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>128</v>
-      </c>
-      <c r="B5" t="s">
-        <v>129</v>
-      </c>
-      <c r="C5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>131</v>
-      </c>
-      <c r="B6" t="s">
-        <v>132</v>
-      </c>
-      <c r="C6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>134</v>
-      </c>
-      <c r="B7" t="s">
-        <v>135</v>
-      </c>
-      <c r="C7" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B8" t="s">
-        <v>138</v>
-      </c>
-      <c r="C8" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>140</v>
-      </c>
-      <c r="B9" t="s">
-        <v>141</v>
-      </c>
-      <c r="C9" t="s">
-        <v>142</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C9" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{5e625f8d-0b53-4f56-9e46-19fa14bb2e5c}" enabled="0" method="" siteId="{5e625f8d-0b53-4f56-9e46-19fa14bb2e5c}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Updated code for service area map
</commit_message>
<xml_diff>
--- a/data/marketplace/MarketplaceBrochureFormularyData.xlsx
+++ b/data/marketplace/MarketplaceBrochureFormularyData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molinahealthcare-my.sharepoint.com/personal/naresh_jangid_molinahealthcare_com/Documents/Automation/molina_automation/marketplace/data/marketplace/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_00DF86192339FA6CDC610236489088D5A02C51E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA811E6E-F4FF-48E2-B8B3-3FAFC50D91F0}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_00DF86192339FA6CDC610236489088D5A02C51E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08557E9C-677D-49DA-B95D-2D99205E5906}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -97,9 +97,6 @@
     <t>2027</t>
   </si>
   <si>
-    <t>CAFormulary27</t>
-  </si>
-  <si>
     <t>CAFormulary27.pdf</t>
   </si>
   <si>
@@ -356,6 +353,9 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>CAFormulary27 - Marketplace 2027</t>
   </si>
 </sst>
 </file>
@@ -816,7 +816,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>111</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
         <v>22</v>
@@ -828,451 +828,451 @@
         <v>24</v>
       </c>
       <c r="E2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" t="s">
         <v>25</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" t="s">
         <v>26</v>
       </c>
-      <c r="G2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>27</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>28</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M2" t="s">
         <v>29</v>
       </c>
-      <c r="K2" t="s">
-        <v>29</v>
-      </c>
-      <c r="L2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>30</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>31</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R2" t="s">
         <v>32</v>
       </c>
-      <c r="P2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>32</v>
-      </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>33</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>34</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>35</v>
-      </c>
-      <c r="U2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
         <v>37</v>
-      </c>
-      <c r="C3" t="s">
-        <v>38</v>
       </c>
       <c r="D3" t="s">
         <v>24</v>
       </c>
       <c r="E3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" t="s">
         <v>39</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" t="s">
         <v>40</v>
       </c>
-      <c r="G3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>41</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>42</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
+        <v>42</v>
+      </c>
+      <c r="L3" t="s">
+        <v>42</v>
+      </c>
+      <c r="M3" t="s">
         <v>43</v>
       </c>
-      <c r="K3" t="s">
-        <v>43</v>
-      </c>
-      <c r="L3" t="s">
-        <v>43</v>
-      </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>44</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>45</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>45</v>
+      </c>
+      <c r="R3" t="s">
         <v>46</v>
       </c>
-      <c r="P3" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>46</v>
-      </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>47</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>48</v>
       </c>
-      <c r="T3" t="s">
-        <v>49</v>
-      </c>
       <c r="U3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" t="s">
         <v>50</v>
-      </c>
-      <c r="C4" t="s">
-        <v>51</v>
       </c>
       <c r="D4" t="s">
         <v>24</v>
       </c>
       <c r="E4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" t="s">
         <v>52</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H4" t="s">
         <v>53</v>
       </c>
-      <c r="G4" t="s">
-        <v>53</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>54</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>55</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
+        <v>55</v>
+      </c>
+      <c r="L4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M4" t="s">
         <v>56</v>
       </c>
-      <c r="K4" t="s">
-        <v>56</v>
-      </c>
-      <c r="L4" t="s">
-        <v>56</v>
-      </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>57</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>58</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>58</v>
+      </c>
+      <c r="R4" t="s">
         <v>59</v>
       </c>
-      <c r="P4" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>59</v>
-      </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>60</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>61</v>
       </c>
-      <c r="T4" t="s">
-        <v>62</v>
-      </c>
       <c r="U4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>110</v>
       </c>
       <c r="B5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" t="s">
         <v>63</v>
-      </c>
-      <c r="C5" t="s">
-        <v>64</v>
       </c>
       <c r="D5" t="s">
         <v>24</v>
       </c>
       <c r="E5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" t="s">
         <v>65</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
+        <v>65</v>
+      </c>
+      <c r="H5" t="s">
         <v>66</v>
       </c>
-      <c r="G5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>67</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>68</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
+        <v>68</v>
+      </c>
+      <c r="L5" t="s">
+        <v>68</v>
+      </c>
+      <c r="M5" t="s">
         <v>69</v>
       </c>
-      <c r="K5" t="s">
-        <v>69</v>
-      </c>
-      <c r="L5" t="s">
-        <v>69</v>
-      </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>70</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>71</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>71</v>
+      </c>
+      <c r="R5" t="s">
         <v>72</v>
       </c>
-      <c r="P5" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>72</v>
-      </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>73</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>74</v>
       </c>
-      <c r="T5" t="s">
-        <v>75</v>
-      </c>
       <c r="U5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" t="s">
         <v>76</v>
-      </c>
-      <c r="C6" t="s">
-        <v>77</v>
       </c>
       <c r="D6" t="s">
         <v>24</v>
       </c>
       <c r="E6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6" t="s">
         <v>78</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H6" t="s">
         <v>79</v>
       </c>
-      <c r="G6" t="s">
-        <v>79</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>80</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>81</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
+        <v>81</v>
+      </c>
+      <c r="L6" t="s">
+        <v>81</v>
+      </c>
+      <c r="M6" t="s">
         <v>82</v>
       </c>
-      <c r="K6" t="s">
-        <v>82</v>
-      </c>
-      <c r="L6" t="s">
-        <v>82</v>
-      </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>83</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>84</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>84</v>
+      </c>
+      <c r="R6" t="s">
         <v>85</v>
       </c>
-      <c r="P6" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>85</v>
-      </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>86</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>87</v>
       </c>
-      <c r="T6" t="s">
-        <v>88</v>
-      </c>
       <c r="U6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" t="s">
         <v>89</v>
-      </c>
-      <c r="C7" t="s">
-        <v>90</v>
       </c>
       <c r="D7" t="s">
         <v>24</v>
       </c>
       <c r="E7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J7" t="s">
+        <v>90</v>
+      </c>
+      <c r="K7" t="s">
+        <v>90</v>
+      </c>
+      <c r="L7" t="s">
+        <v>90</v>
+      </c>
+      <c r="M7" t="s">
         <v>91</v>
       </c>
-      <c r="K7" t="s">
-        <v>91</v>
-      </c>
-      <c r="L7" t="s">
-        <v>91</v>
-      </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>92</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>93</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>93</v>
+      </c>
+      <c r="R7" t="s">
         <v>94</v>
       </c>
-      <c r="P7" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>94</v>
-      </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>95</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
+        <v>35</v>
+      </c>
+      <c r="U7" t="s">
         <v>96</v>
-      </c>
-      <c r="T7" t="s">
-        <v>36</v>
-      </c>
-      <c r="U7" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" t="s">
         <v>98</v>
-      </c>
-      <c r="C8" t="s">
-        <v>99</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
       </c>
       <c r="E8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F8" t="s">
         <v>100</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>100</v>
+      </c>
+      <c r="H8" t="s">
         <v>101</v>
       </c>
-      <c r="G8" t="s">
-        <v>101</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>102</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>103</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
+        <v>103</v>
+      </c>
+      <c r="L8" t="s">
+        <v>103</v>
+      </c>
+      <c r="M8" t="s">
         <v>104</v>
       </c>
-      <c r="K8" t="s">
-        <v>104</v>
-      </c>
-      <c r="L8" t="s">
-        <v>104</v>
-      </c>
-      <c r="M8" t="s">
+      <c r="N8" t="s">
         <v>105</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>106</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>106</v>
+      </c>
+      <c r="R8" t="s">
         <v>107</v>
       </c>
-      <c r="P8" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>107</v>
-      </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>108</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>109</v>
       </c>
-      <c r="T8" t="s">
-        <v>110</v>
-      </c>
       <c r="U8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:U1 B4:U8 B3:U3 B2:U2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:U1 B4:U8 B3:U3 B2:D2 F2:U2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Consolidate logs into utils/logs; add plan search specs and split SOB report script
</commit_message>
<xml_diff>
--- a/data/marketplace/MarketplaceBrochureFormularyData.xlsx
+++ b/data/marketplace/MarketplaceBrochureFormularyData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molinahealthcare-my.sharepoint.com/personal/naresh_jangid_molinahealthcare_com/Documents/Automation/molina_automation/marketplace/data/marketplace/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molinahealthcare-my.sharepoint.com/personal/seeram_tarunvardhan_molinahealthcare_com/Documents/Desktop/Automationss/IMP/marketplace/data/marketplace/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_00DF86192339FA6CDC610236489088D5A02C51E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08557E9C-677D-49DA-B95D-2D99205E5906}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="11_00DF86192339FA6CDC610236489088D5A02C51E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E1C57D9-DDED-4B0C-A08B-BA5EF931ACAF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BrochureFormulary" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="113">
   <si>
     <t>Run</t>
   </si>
@@ -190,21 +190,6 @@
     <t>NM Plan Brochure</t>
   </si>
   <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/brochure/2027/english/NMMBRBrochure27.pdf</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/brochure/2027/spanish/NMMBRBrochure27.pdf</t>
-  </si>
-  <si>
-    <t>NM Broker Brochure</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/brochure/2027/english/NMBrochure27.pdf</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/brochure/2027/spanish/NMBrochure27.pdf</t>
-  </si>
-  <si>
     <t>MolinaHealthcare.com/NMFormulary27</t>
   </si>
   <si>
@@ -356,6 +341,24 @@
   </si>
   <si>
     <t>CAFormulary27 - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/Project/PWS/Healthcare/PDF/PDF/IFP/NM/Materials/brochure/2027/English/NMBrochure27.pdf</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/Project/PWS/Healthcare/PDF/PDF/IFP/NM/Materials/brochure/2027/Spanish/NMBrochure27.pdf</t>
+  </si>
+  <si>
+    <t>NM Plan Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/Project/PWS/Healthcare/PDF/PDF/IFP/NM/Materials/brochure/2027/English/NMMBRBrochure27.pdf</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/Project/PWS/Healthcare/PDF/PDF/IFP/NM/Materials/brochure/2027/Spanish/NMMBRBrochure27.pdf</t>
+  </si>
+  <si>
+    <t>NM Broker Brochure - Marketplace 2027</t>
   </si>
 </sst>
 </file>
@@ -408,6 +411,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -733,23 +740,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U8"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.796875" customWidth="1"/>
+    <col min="1" max="1" width="9.83203125" customWidth="1"/>
     <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.796875" customWidth="1"/>
-    <col min="4" max="4" width="10.796875" customWidth="1"/>
-    <col min="5" max="7" width="30.796875" customWidth="1"/>
-    <col min="8" max="9" width="110.796875" customWidth="1"/>
-    <col min="10" max="12" width="30.796875" customWidth="1"/>
-    <col min="13" max="14" width="110.796875" customWidth="1"/>
-    <col min="15" max="17" width="30.796875" customWidth="1"/>
-    <col min="18" max="19" width="110.796875" customWidth="1"/>
-    <col min="20" max="20" width="40.796875" customWidth="1"/>
-    <col min="21" max="21" width="46.796875" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="7" width="30.83203125" customWidth="1"/>
+    <col min="8" max="9" width="110.83203125" customWidth="1"/>
+    <col min="10" max="12" width="30.83203125" customWidth="1"/>
+    <col min="13" max="14" width="110.83203125" customWidth="1"/>
+    <col min="15" max="17" width="30.83203125" customWidth="1"/>
+    <col min="18" max="19" width="110.83203125" customWidth="1"/>
+    <col min="20" max="20" width="40.83203125" customWidth="1"/>
+    <col min="21" max="21" width="46.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -814,9 +821,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>105</v>
       </c>
       <c r="B2" t="s">
         <v>22</v>
@@ -828,7 +835,7 @@
         <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="F2" t="s">
         <v>25</v>
@@ -879,9 +886,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B3" t="s">
         <v>36</v>
@@ -944,9 +951,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
         <v>49</v>
@@ -976,178 +983,178 @@
         <v>55</v>
       </c>
       <c r="K4" t="s">
-        <v>55</v>
+        <v>109</v>
       </c>
       <c r="L4" t="s">
-        <v>55</v>
+        <v>109</v>
       </c>
       <c r="M4" t="s">
+        <v>110</v>
+      </c>
+      <c r="N4" t="s">
+        <v>111</v>
+      </c>
+      <c r="O4" t="s">
+        <v>112</v>
+      </c>
+      <c r="P4" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>112</v>
+      </c>
+      <c r="R4" t="s">
+        <v>107</v>
+      </c>
+      <c r="S4" t="s">
+        <v>108</v>
+      </c>
+      <c r="T4" t="s">
         <v>56</v>
-      </c>
-      <c r="N4" t="s">
-        <v>57</v>
-      </c>
-      <c r="O4" t="s">
-        <v>58</v>
-      </c>
-      <c r="P4" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>58</v>
-      </c>
-      <c r="R4" t="s">
-        <v>59</v>
-      </c>
-      <c r="S4" t="s">
-        <v>60</v>
-      </c>
-      <c r="T4" t="s">
-        <v>61</v>
       </c>
       <c r="U4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
         <v>24</v>
       </c>
       <c r="E5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>60</v>
+      </c>
+      <c r="H5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" t="s">
+        <v>62</v>
+      </c>
+      <c r="J5" t="s">
+        <v>63</v>
+      </c>
+      <c r="K5" t="s">
+        <v>63</v>
+      </c>
+      <c r="L5" t="s">
+        <v>63</v>
+      </c>
+      <c r="M5" t="s">
         <v>64</v>
       </c>
-      <c r="F5" t="s">
+      <c r="N5" t="s">
         <v>65</v>
       </c>
-      <c r="G5" t="s">
-        <v>65</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="O5" t="s">
         <v>66</v>
       </c>
-      <c r="I5" t="s">
+      <c r="P5" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>66</v>
+      </c>
+      <c r="R5" t="s">
         <v>67</v>
       </c>
-      <c r="J5" t="s">
+      <c r="S5" t="s">
         <v>68</v>
       </c>
-      <c r="K5" t="s">
-        <v>68</v>
-      </c>
-      <c r="L5" t="s">
-        <v>68</v>
-      </c>
-      <c r="M5" t="s">
+      <c r="T5" t="s">
         <v>69</v>
-      </c>
-      <c r="N5" t="s">
-        <v>70</v>
-      </c>
-      <c r="O5" t="s">
-        <v>71</v>
-      </c>
-      <c r="P5" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>71</v>
-      </c>
-      <c r="R5" t="s">
-        <v>72</v>
-      </c>
-      <c r="S5" t="s">
-        <v>73</v>
-      </c>
-      <c r="T5" t="s">
-        <v>74</v>
       </c>
       <c r="U5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="D6" t="s">
         <v>24</v>
       </c>
       <c r="E6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I6" t="s">
+        <v>75</v>
+      </c>
+      <c r="J6" t="s">
+        <v>76</v>
+      </c>
+      <c r="K6" t="s">
+        <v>76</v>
+      </c>
+      <c r="L6" t="s">
+        <v>76</v>
+      </c>
+      <c r="M6" t="s">
         <v>77</v>
       </c>
-      <c r="F6" t="s">
+      <c r="N6" t="s">
         <v>78</v>
       </c>
-      <c r="G6" t="s">
-        <v>78</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="O6" t="s">
         <v>79</v>
       </c>
-      <c r="I6" t="s">
+      <c r="P6" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>79</v>
+      </c>
+      <c r="R6" t="s">
         <v>80</v>
       </c>
-      <c r="J6" t="s">
+      <c r="S6" t="s">
         <v>81</v>
       </c>
-      <c r="K6" t="s">
-        <v>81</v>
-      </c>
-      <c r="L6" t="s">
-        <v>81</v>
-      </c>
-      <c r="M6" t="s">
+      <c r="T6" t="s">
         <v>82</v>
-      </c>
-      <c r="N6" t="s">
-        <v>83</v>
-      </c>
-      <c r="O6" t="s">
-        <v>84</v>
-      </c>
-      <c r="P6" t="s">
-        <v>84</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>84</v>
-      </c>
-      <c r="R6" t="s">
-        <v>85</v>
-      </c>
-      <c r="S6" t="s">
-        <v>86</v>
-      </c>
-      <c r="T6" t="s">
-        <v>87</v>
       </c>
       <c r="U6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C7" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D7" t="s">
         <v>24</v>
@@ -1168,102 +1175,102 @@
         <v>35</v>
       </c>
       <c r="J7" t="s">
+        <v>85</v>
+      </c>
+      <c r="K7" t="s">
+        <v>85</v>
+      </c>
+      <c r="L7" t="s">
+        <v>85</v>
+      </c>
+      <c r="M7" t="s">
+        <v>86</v>
+      </c>
+      <c r="N7" t="s">
+        <v>87</v>
+      </c>
+      <c r="O7" t="s">
+        <v>88</v>
+      </c>
+      <c r="P7" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>88</v>
+      </c>
+      <c r="R7" t="s">
+        <v>89</v>
+      </c>
+      <c r="S7" t="s">
         <v>90</v>
-      </c>
-      <c r="K7" t="s">
-        <v>90</v>
-      </c>
-      <c r="L7" t="s">
-        <v>90</v>
-      </c>
-      <c r="M7" t="s">
-        <v>91</v>
-      </c>
-      <c r="N7" t="s">
-        <v>92</v>
-      </c>
-      <c r="O7" t="s">
-        <v>93</v>
-      </c>
-      <c r="P7" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>93</v>
-      </c>
-      <c r="R7" t="s">
-        <v>94</v>
-      </c>
-      <c r="S7" t="s">
-        <v>95</v>
       </c>
       <c r="T7" t="s">
         <v>35</v>
       </c>
       <c r="U7" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B8" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C8" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
       </c>
       <c r="E8" t="s">
+        <v>94</v>
+      </c>
+      <c r="F8" t="s">
+        <v>95</v>
+      </c>
+      <c r="G8" t="s">
+        <v>95</v>
+      </c>
+      <c r="H8" t="s">
+        <v>96</v>
+      </c>
+      <c r="I8" t="s">
+        <v>97</v>
+      </c>
+      <c r="J8" t="s">
+        <v>98</v>
+      </c>
+      <c r="K8" t="s">
+        <v>98</v>
+      </c>
+      <c r="L8" t="s">
+        <v>98</v>
+      </c>
+      <c r="M8" t="s">
         <v>99</v>
       </c>
-      <c r="F8" t="s">
+      <c r="N8" t="s">
         <v>100</v>
       </c>
-      <c r="G8" t="s">
-        <v>100</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="O8" t="s">
         <v>101</v>
       </c>
-      <c r="I8" t="s">
+      <c r="P8" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>101</v>
+      </c>
+      <c r="R8" t="s">
         <v>102</v>
       </c>
-      <c r="J8" t="s">
+      <c r="S8" t="s">
         <v>103</v>
       </c>
-      <c r="K8" t="s">
-        <v>103</v>
-      </c>
-      <c r="L8" t="s">
-        <v>103</v>
-      </c>
-      <c r="M8" t="s">
+      <c r="T8" t="s">
         <v>104</v>
-      </c>
-      <c r="N8" t="s">
-        <v>105</v>
-      </c>
-      <c r="O8" t="s">
-        <v>106</v>
-      </c>
-      <c r="P8" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>106</v>
-      </c>
-      <c r="R8" t="s">
-        <v>107</v>
-      </c>
-      <c r="S8" t="s">
-        <v>108</v>
-      </c>
-      <c r="T8" t="s">
-        <v>109</v>
       </c>
       <c r="U8" t="s">
         <v>35</v>
@@ -1272,7 +1279,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:U1 B4:U8 B3:U3 B2:D2 F2:U2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:U1 B5:U8 B3:U3 B2:D2 F2:U2 B4:J4 T4:U4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add 2027 Drug Lookup Tool automation suite (EN/ES, CDP attach, dashboards) + marketplace updates
</commit_message>
<xml_diff>
--- a/data/marketplace/MarketplaceBrochureFormularyData.xlsx
+++ b/data/marketplace/MarketplaceBrochureFormularyData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molinahealthcare-my.sharepoint.com/personal/seeram_tarunvardhan_molinahealthcare_com/Documents/Desktop/Automationss/IMP/marketplace/data/marketplace/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="11_00DF86192339FA6CDC610236489088D5A02C51E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E1C57D9-DDED-4B0C-A08B-BA5EF931ACAF}"/>
+  <xr:revisionPtr revIDLastSave="172" documentId="11_00DF86192339FA6CDC610236489088D5A02C51E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D85B77EE-35D8-4F19-BE44-F84063185B79}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="125">
   <si>
     <t>Run</t>
   </si>
@@ -359,6 +359,42 @@
   </si>
   <si>
     <t>NM Broker Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>TX Broker Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>TX Off Exchange Broker Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>TX Off Exchange Plan Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>TX Plan Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>CA Plan Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>CA Broker Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>NV Plan Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>NV Broker Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>ID Broker Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>ID Plan Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>WA Plan Brochure - Marketplace 2027</t>
+  </si>
+  <si>
+    <t>WA Broker Brochure - Marketplace 2027</t>
   </si>
 </sst>
 </file>
@@ -411,10 +447,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -823,7 +855,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
         <v>22</v>
@@ -853,10 +885,10 @@
         <v>28</v>
       </c>
       <c r="K2" t="s">
-        <v>28</v>
+        <v>117</v>
       </c>
       <c r="L2" t="s">
-        <v>28</v>
+        <v>117</v>
       </c>
       <c r="M2" t="s">
         <v>29</v>
@@ -868,10 +900,10 @@
         <v>31</v>
       </c>
       <c r="P2" t="s">
-        <v>31</v>
+        <v>118</v>
       </c>
       <c r="Q2" t="s">
-        <v>31</v>
+        <v>118</v>
       </c>
       <c r="R2" t="s">
         <v>32</v>
@@ -888,7 +920,7 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
         <v>36</v>
@@ -918,10 +950,10 @@
         <v>42</v>
       </c>
       <c r="K3" t="s">
-        <v>42</v>
+        <v>122</v>
       </c>
       <c r="L3" t="s">
-        <v>42</v>
+        <v>122</v>
       </c>
       <c r="M3" t="s">
         <v>43</v>
@@ -933,10 +965,10 @@
         <v>45</v>
       </c>
       <c r="P3" t="s">
-        <v>45</v>
+        <v>121</v>
       </c>
       <c r="Q3" t="s">
-        <v>45</v>
+        <v>121</v>
       </c>
       <c r="R3" t="s">
         <v>46</v>
@@ -953,7 +985,7 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>105</v>
       </c>
       <c r="B4" t="s">
         <v>49</v>
@@ -1018,7 +1050,7 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>105</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
         <v>57</v>
@@ -1048,10 +1080,10 @@
         <v>63</v>
       </c>
       <c r="K5" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="L5" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="M5" t="s">
         <v>64</v>
@@ -1063,10 +1095,10 @@
         <v>66</v>
       </c>
       <c r="P5" t="s">
-        <v>66</v>
+        <v>120</v>
       </c>
       <c r="Q5" t="s">
-        <v>66</v>
+        <v>120</v>
       </c>
       <c r="R5" t="s">
         <v>67</v>
@@ -1113,10 +1145,10 @@
         <v>76</v>
       </c>
       <c r="K6" t="s">
-        <v>76</v>
+        <v>116</v>
       </c>
       <c r="L6" t="s">
-        <v>76</v>
+        <v>116</v>
       </c>
       <c r="M6" t="s">
         <v>77</v>
@@ -1128,10 +1160,10 @@
         <v>79</v>
       </c>
       <c r="P6" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="Q6" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="R6" t="s">
         <v>80</v>
@@ -1165,12 +1197,6 @@
       <c r="F7" t="s">
         <v>35</v>
       </c>
-      <c r="G7" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7" t="s">
-        <v>35</v>
-      </c>
       <c r="I7" t="s">
         <v>35</v>
       </c>
@@ -1178,10 +1204,10 @@
         <v>85</v>
       </c>
       <c r="K7" t="s">
-        <v>85</v>
+        <v>115</v>
       </c>
       <c r="L7" t="s">
-        <v>85</v>
+        <v>115</v>
       </c>
       <c r="M7" t="s">
         <v>86</v>
@@ -1193,10 +1219,10 @@
         <v>88</v>
       </c>
       <c r="P7" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="Q7" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="R7" t="s">
         <v>89</v>
@@ -1213,7 +1239,7 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>105</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
         <v>92</v>
@@ -1243,10 +1269,10 @@
         <v>98</v>
       </c>
       <c r="K8" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L8" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="M8" t="s">
         <v>99</v>
@@ -1258,10 +1284,10 @@
         <v>101</v>
       </c>
       <c r="P8" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="Q8" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="R8" t="s">
         <v>102</v>
@@ -1279,7 +1305,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:U1 B5:U8 B3:U3 B2:D2 F2:U2 B4:J4 T4:U4" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:U1 B5:J5 B3:J3 B2:D2 F2:J2 B4:J4 T4:U4 B8:J8 B6:J6 T6:U6 B7:F7 T7:U7 O7 O6 I7:J7 O2 T2:U2 O5 R5:U5 T3:U3 O3 O8 T8:U8" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>